<commit_message>
final changes, layout changed using treeview, added average score
</commit_message>
<xml_diff>
--- a/student_scores.xlsx
+++ b/student_scores.xlsx
@@ -9,7 +9,7 @@
     <sheet name="ScoreTracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,30 +435,109 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>kevin</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Failed</t>
-        </is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F2">
+        <f>AVERAGE(B2:B1000)</f>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kenneth</t>
+          <t>Tung Tung Sahur</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ballerina</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>99</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bagsak to</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>56</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>huhu</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>88</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>jjj</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>87</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>pampababa ng ave</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>23</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
     </row>

</xml_diff>